<commit_message>
replace hardcoded TP with notation catalogue
</commit_message>
<xml_diff>
--- a/inst/CPions_TP_formula.xlsx
+++ b/inst/CPions_TP_formula.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
   <si>
     <t xml:space="preserve">Name of TP</t>
   </si>
@@ -150,30 +150,6 @@
   </si>
   <si>
     <t xml:space="preserve">C10H14Cl6O2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Br-hydroxylation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-Br+OH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CxH2x+2-y-z+1ClyBrz-1O</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C10H16Cl4Br2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C10H17Cl4BrO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Double Br-hydroxylation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-2Br+2OH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CxH2x+2-y-z+2ClyBrz-2O2</t>
   </si>
   <si>
     <t xml:space="preserve">Methoxylation</t>
@@ -795,40 +771,40 @@
         <v>48</v>
       </c>
       <c r="D11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" t="s">
         <v>49</v>
       </c>
-      <c r="E11" t="s">
-        <v>50</v>
-      </c>
       <c r="F11" t="s">
         <v>11</v>
       </c>
       <c r="G11" t="n">
-        <v>370.9144</v>
+        <v>374.9416</v>
       </c>
       <c r="H11"/>
     </row>
     <row r="12">
       <c r="A12" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" t="s">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>52</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" t="s">
         <v>53</v>
       </c>
-      <c r="D12" t="s">
-        <v>49</v>
-      </c>
-      <c r="E12" t="s">
-        <v>25</v>
-      </c>
       <c r="F12" t="s">
         <v>11</v>
       </c>
       <c r="G12" t="n">
-        <v>308.9988</v>
+        <v>340.9806</v>
       </c>
       <c r="H12"/>
     </row>
@@ -852,57 +828,9 @@
         <v>11</v>
       </c>
       <c r="G13" t="n">
-        <v>374.9416</v>
+        <v>372.8896</v>
       </c>
       <c r="H13"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" t="s">
-        <v>10</v>
-      </c>
-      <c r="E14" t="s">
-        <v>61</v>
-      </c>
-      <c r="F14" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" t="n">
-        <v>340.9806</v>
-      </c>
-      <c r="H14"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" t="s">
-        <v>65</v>
-      </c>
-      <c r="F15" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" t="n">
-        <v>372.8896</v>
-      </c>
-      <c r="H15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>